<commit_message>
Wochenplan aktualisiert + Planner fixes
</commit_message>
<xml_diff>
--- a/Wochenplan/Wochenuebersicht_20260519.xlsx
+++ b/Wochenplan/Wochenuebersicht_20260519.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Produktionsbedarf" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Wochenplan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produktionsbedarf" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wochenplan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -629,13 +629,13 @@
         <v>9</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>0</v>
@@ -657,13 +657,13 @@
         <v>11</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>0</v>
@@ -685,10 +685,10 @@
         <v>9</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G6" s="6" t="n">
         <v>12</v>
@@ -741,20 +741,20 @@
         <v>18</v>
       </c>
       <c r="E8" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="F8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="H8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Beide ueber Schwelle - keine Produktion</t>
+          <t>Beeren unter Schwelle (32.0&lt;45)</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
         <v>18</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>0</v>
@@ -787,7 +787,7 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Beide ueber Schwelle - keine Produktion</t>
+          <t>Beeren unter Schwelle (32.0&lt;45)</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
         <v>20</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0</v>
@@ -822,7 +822,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Lager OK (40&gt;=30)</t>
+          <t>Lager OK (50&gt;=30)</t>
         </is>
       </c>
     </row>
@@ -840,11 +840,11 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3840g</t>
+          <t>7800g</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>12x/2400g</t>
+          <t>18x/3600g</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,19 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>8x/1440g</t>
+          <t>10x/1800g</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tartelette:</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>60x/2400g</t>
         </is>
       </c>
     </row>
@@ -887,7 +899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -942,7 +954,7 @@
       <c r="C4" s="14" t="inlineStr"/>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>Alle Boeden: 12x 30x20 Schnitte, 8x Murbeteig rund + 4x Murbeteig rund fuer naechsten Montag</t>
+          <t>Alle Boeden: 18x 30x20 Schnitte, 10x Murbeteig rund, 60x Tartelette + 4x Murbeteig rund fuer naechsten Montag</t>
         </is>
       </c>
     </row>
@@ -958,7 +970,7 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Charge 1/4</t>
+          <t>Charge 1/5</t>
         </is>
       </c>
     </row>
@@ -974,7 +986,7 @@
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>Charge 2/4</t>
+          <t>Charge 2/5</t>
         </is>
       </c>
     </row>
@@ -995,32 +1007,41 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr"/>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Kaese-Rhabarber Schnitte</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Charge 1/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>MITTWOCH</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="14" t="inlineStr"/>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Bienenstich</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>Charge 2/2</t>
-        </is>
-      </c>
-    </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>DONNERSTAG</t>
+      <c r="A10" s="14" t="inlineStr"/>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Kaesekuchen</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Charge 3/5</t>
         </is>
       </c>
     </row>
@@ -1028,22 +1049,31 @@
       <c r="A11" s="14" t="inlineStr"/>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Donauwelle</t>
+          <t>Kaesekuchen</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
+          <t>Charge 4/5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="14" t="inlineStr"/>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Lauch-Speck Quiche</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
           <t>Charge 1/1</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>FREITAG</t>
         </is>
       </c>
     </row>
@@ -1051,31 +1081,22 @@
       <c r="A13" s="14" t="inlineStr"/>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>Kaesekuchen</t>
+          <t>Beeren Tartelette</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>Charge 3/4</t>
+          <t>60 Stueck</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="14" t="inlineStr"/>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>Kaesekuchen</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Charge 4/4</t>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>DONNERSTAG</t>
         </is>
       </c>
     </row>
@@ -1083,15 +1104,15 @@
       <c r="A15" s="14" t="inlineStr"/>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Lauch-Speck Quiche</t>
+          <t>Kaesekuchen</t>
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Charge 1/1</t>
+          <t>Charge 5/5</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1120,7 @@
       <c r="A16" s="14" t="inlineStr"/>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Kaese-Rhabarber Schnitte</t>
+          <t>Donauwelle</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
@@ -1108,16 +1129,55 @@
       <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Charge 1/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>FREITAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="14" t="inlineStr"/>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Bienenstich</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Charge 2/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="14" t="inlineStr"/>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Kaese-Rhabarber Schnitte</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>Charge 2/2</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A9:D9"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>